<commit_message>
Live demo at life-crm.jerryfane.com
- demo/build.py bundles a landing page, Maya's site + CV, her dashboard, and the finance and health dashboards
- demo/wrangler.json: one Worker on the custom domain, no workers.dev or preview URLs
- robots.txt keeps the fictional pages out of search; landing page stays indexable
- examples: replace a real-sounding hospital name with a made-up one

Closes #3
</commit_message>
<xml_diff>
--- a/examples/career/crm.xlsx
+++ b/examples/career/crm.xlsx
@@ -5015,22 +5015,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ospedale San Marco</t>
+          <t>Hospital Costa Clara</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Turin</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Dermatology</t>
+          <t>Family Medicine</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>National exam</t>
+          <t>MIR exam</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Profile compact: one-line sections (certificates, languages) on the site and CV
- Profile 'compact' lists Entries sections shown one line per row; a title+summary row shows as 'Title: summary'
- Maya's Certifications use it
</commit_message>
<xml_diff>
--- a/examples/career/crm.xlsx
+++ b/examples/career/crm.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -573,6 +573,18 @@
       <c r="B11" s="2" t="inlineStr">
         <is>
           <t>https://life-crm.jerryfane.com/demo/site</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Certifications</t>
         </is>
       </c>
     </row>

</xml_diff>